<commit_message>
Fixed planning section for single buyer article number not displaying plant name correctly.
</commit_message>
<xml_diff>
--- a/zlpi.xlsx
+++ b/zlpi.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CW27/26</t>
+          <t>CW38/26</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -597,7 +597,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CW36/26</t>
+          <t>CW38/26</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -640,7 +640,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CW37/26</t>
+          <t>CW38/26</t>
         </is>
       </c>
       <c r="I5" t="n">

</xml_diff>

<commit_message>
Dashboard added, new style for upper menu.
</commit_message>
<xml_diff>
--- a/zlpi.xlsx
+++ b/zlpi.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CW38/26</t>
+          <t>CW27/26</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -597,7 +597,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CW38/26</t>
+          <t>CW36/26</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -640,7 +640,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CW38/26</t>
+          <t>CW37/26</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1877,17 +1877,17 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2027-04-12</t>
+          <t>2027-02-22</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>CW15/27</t>
+          <t>CW08/27</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>CW13/27</t>
+          <t>CW06/27</t>
         </is>
       </c>
       <c r="I34" t="n">
@@ -1920,17 +1920,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2027-04-12</t>
+          <t>2027-02-22</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>CW15/27</t>
+          <t>CW08/27</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>CW13/27</t>
+          <t>CW06/27</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -1959,21 +1959,21 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>7680</v>
+        <v>3840</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2027-06-28</t>
+          <t>2027-04-19</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>CW26/27</t>
+          <t>CW16/27</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>CW24/27</t>
+          <t>CW14/27</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-12-28</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">

</xml_diff>

<commit_message>
Added Safety stock functionality.
</commit_message>
<xml_diff>
--- a/zlpi.xlsx
+++ b/zlpi.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1536</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="6">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1536</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="7">
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>3072</v>
+        <v>3075</v>
       </c>
     </row>
     <row r="8">
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1920</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="9">
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2688</v>
+        <v>2829</v>
       </c>
     </row>
     <row r="10">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2304</v>
+        <v>2337</v>
       </c>
     </row>
     <row r="11">
@@ -902,7 +902,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>768</v>
+        <v>861</v>
       </c>
     </row>
     <row r="12">
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1536</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="13">
@@ -988,7 +988,7 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>1536</v>
+        <v>1599</v>
       </c>
     </row>
     <row r="14">
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2304</v>
+        <v>2337</v>
       </c>
     </row>
     <row r="15">
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>768</v>
+        <v>738</v>
       </c>
     </row>
     <row r="16">
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>240</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>2160</v>
+        <v>2351</v>
       </c>
     </row>
     <row r="24">
@@ -1461,7 +1461,7 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>3840</v>
+        <v>3649</v>
       </c>
     </row>
     <row r="25">
@@ -1590,7 +1590,7 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>381</v>
+        <v>572</v>
       </c>
     </row>
     <row r="28">
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>720</v>
+        <v>388</v>
       </c>
     </row>
     <row r="29">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>699</v>
+        <v>825</v>
       </c>
     </row>
     <row r="33">
@@ -1934,7 +1934,7 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>3468</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="36">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>2135</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="37">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>5500001821</t>
+          <t>5500001822</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1998,29 +1998,29 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>F-804661.03-3005-A.AU.KL</t>
+          <t>F-804661-3005-A.IR.KL</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>3432</v>
+        <v>3840</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2027-04-19</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>CW53/26</t>
+          <t>CW16/27</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>CW51/26</t>
+          <t>CW14/27</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>3432</v>
+        <v>2130</v>
       </c>
     </row>
     <row r="38">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>5500001821</t>
+          <t>5500001822</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2041,29 +2041,29 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>F-804661.03-3005-A.AU.KL</t>
+          <t>F-804661-3005-A.IR.KL</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>3432</v>
+        <v>3840</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2027-04-12</t>
+          <t>2027-08-01</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>CW15/27</t>
+          <t>CW30/27</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>CW13/27</t>
+          <t>CW28/27</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>3432</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39">
@@ -2088,24 +2088,110 @@
         </is>
       </c>
       <c r="E39" t="n">
+        <v>3432</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>CW53/26</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>CW51/26</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>3432</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER PORTUGAL</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>5500001821</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>F-804661.03-3005-A.AU.KL</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>3432</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2027-04-12</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>CW15/27</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>CW13/27</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>3432</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER PORTUGAL</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>5500001821</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>F-804661.03-3005-A.AU.KL</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
         <v>8580</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>2027-06-28</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>CW26/27</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>CW24/27</t>
         </is>
       </c>
-      <c r="I39" t="n">
+      <c r="I41" t="n">
         <v>2960</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard updated with lists of delayed orders and orders needed.
</commit_message>
<xml_diff>
--- a/zlpi.xlsx
+++ b/zlpi.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CW27/26</t>
+          <t>CW37/26</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -597,7 +597,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CW36/26</t>
+          <t>CW37/26</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>1710</v>
+        <v>377</v>
       </c>
     </row>
     <row r="37">
@@ -2020,7 +2020,7 @@
         </is>
       </c>
       <c r="I37" t="n">
-        <v>2130</v>
+        <v>3463</v>
       </c>
     </row>
     <row r="38">

</xml_diff>

<commit_message>
New style for status bar.
</commit_message>
<xml_diff>
--- a/zlpi.xlsx
+++ b/zlpi.xlsx
@@ -1768,7 +1768,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SCHAEFFLER PORTUGAL</t>
+          <t>SCHAEFFLER PORTUGALLL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1811,7 +1811,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SCHAEFFLER PORTUGAL</t>
+          <t>SCHAEFFLER PORTUGALLL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">

</xml_diff>

<commit_message>
Changes in visual UI.
</commit_message>
<xml_diff>
--- a/zlpi.xlsx
+++ b/zlpi.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,25 +497,25 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1536</v>
+        <v>768</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>CW45/26</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>CW36/26</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>CW37/26</t>
-        </is>
-      </c>
       <c r="I2" t="n">
-        <v>1536</v>
+        <v>768</v>
       </c>
     </row>
     <row r="3">
@@ -540,25 +540,25 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>806</v>
+        <v>1536</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>CW47/26</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>CW38/26</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>CW29/26</t>
-        </is>
-      </c>
       <c r="I3" t="n">
-        <v>806</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="4">
@@ -583,25 +583,25 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>768</v>
+        <v>3840</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CW45/26</t>
+          <t>CW02/27</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CW37/26</t>
+          <t>CW46/26</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>768</v>
+        <v>3840</v>
       </c>
     </row>
     <row r="5">
@@ -626,25 +626,25 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1536</v>
+        <v>3072</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CW46/26</t>
+          <t>CW09/27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CW37/26</t>
+          <t>CW53/26</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1599</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="6">
@@ -669,25 +669,25 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1536</v>
+        <v>3072</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CW04/27</t>
+          <t>CW09/27</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CW48/26</t>
+          <t>CW53/26</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1599</v>
+        <v>384</v>
       </c>
     </row>
     <row r="7">
@@ -712,25 +712,25 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3072</v>
+        <v>1536</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2027-03-25</t>
+          <t>2027-04-23</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CW12/27</t>
+          <t>CW16/27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CW03/27</t>
+          <t>CW07/27</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>3075</v>
+        <v>616</v>
       </c>
     </row>
     <row r="8">
@@ -755,25 +755,25 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>4608</v>
+        <v>1536</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-04-23</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CW17/27</t>
+          <t>CW16/27</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>CW08/27</t>
+          <t>CW07/27</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1791</v>
+        <v>920</v>
       </c>
     </row>
     <row r="9">
@@ -798,25 +798,25 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4608</v>
+        <v>3840</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-06-01</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>CW17/27</t>
+          <t>CW22/27</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>CW08/27</t>
+          <t>CW13/27</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2829</v>
+        <v>3840</v>
       </c>
     </row>
     <row r="10">
@@ -841,25 +841,25 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2304</v>
+        <v>1536</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2027-07-01</t>
+          <t>2027-09-01</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>CW35/27</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>CW26/27</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>CW17/27</t>
-        </is>
-      </c>
       <c r="I10" t="n">
-        <v>2337</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="11">
@@ -884,25 +884,25 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>768</v>
+        <v>2304</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2027-10-01</t>
+          <t>2027-11-01</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CW39/27</t>
+          <t>CW44/27</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CW30/27</t>
+          <t>CW35/27</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>861</v>
+        <v>2304</v>
       </c>
     </row>
     <row r="12">
@@ -931,21 +931,21 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2027-12-01</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>CW48/27</t>
+          <t>CW52/27</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CW39/27</t>
+          <t>CW43/27</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1599</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="13">
@@ -974,21 +974,21 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2028-01-01</t>
+          <t>2028-03-01</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>CW09/28</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>CW52/27</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>CW43/27</t>
-        </is>
-      </c>
       <c r="I13" t="n">
-        <v>1599</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="14">
@@ -1013,25 +1013,25 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2304</v>
+        <v>4663</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2028-03-01</t>
+          <t>2028-05-01</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>CW18/28</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>CW09/28</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>CW52/27</t>
-        </is>
-      </c>
       <c r="I14" t="n">
-        <v>2337</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="15">
@@ -1056,25 +1056,25 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1920</v>
+        <v>4080</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CW36/26</t>
+          <t>CW02/27</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CW27/26</t>
+          <t>CW46/26</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>960</v>
+        <v>2351</v>
       </c>
     </row>
     <row r="16">
@@ -1099,25 +1099,25 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1920</v>
+        <v>4080</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CW36/26</t>
+          <t>CW02/27</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>CW27/26</t>
+          <t>CW46/26</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>960</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="17">
@@ -1142,25 +1142,25 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>3120</v>
+        <v>3360</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CW40/26</t>
+          <t>CW09/27</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>CW31/26</t>
+          <t>CW53/26</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>3120</v>
+        <v>2351</v>
       </c>
     </row>
     <row r="18">
@@ -1185,25 +1185,25 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1440</v>
+        <v>3360</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>CW42/26</t>
+          <t>CW09/27</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>CW33/26</t>
+          <t>CW53/26</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>1440</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="19">
@@ -1228,25 +1228,25 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1440</v>
+        <v>720</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-04-23</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CW04/27</t>
+          <t>CW16/27</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>CW48/26</t>
+          <t>CW07/27</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>1391</v>
+        <v>720</v>
       </c>
     </row>
     <row r="20">
@@ -1271,25 +1271,25 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>1440</v>
+        <v>2160</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2027-01-25</t>
+          <t>2027-06-01</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>CW04/27</t>
+          <t>CW22/27</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CW48/26</t>
+          <t>CW13/27</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>49</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="21">
@@ -1314,25 +1314,25 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1680</v>
+        <v>720</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2027-03-25</t>
+          <t>2027-08-01</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CW12/27</t>
+          <t>CW30/27</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CW03/27</t>
+          <t>CW21/27</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>1680</v>
+        <v>720</v>
       </c>
     </row>
     <row r="22">
@@ -1357,25 +1357,25 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>6000</v>
+        <v>1440</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-09-01</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>CW17/27</t>
+          <t>CW35/27</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CW08/27</t>
+          <t>CW26/27</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>2351</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="23">
@@ -1400,25 +1400,25 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>6000</v>
+        <v>1920</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2027-05-01</t>
+          <t>2027-11-01</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>CW17/27</t>
+          <t>CW44/27</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>CW08/27</t>
+          <t>CW35/27</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>3649</v>
+        <v>332</v>
       </c>
     </row>
     <row r="24">
@@ -1443,25 +1443,25 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1200</v>
+        <v>1920</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2027-08-01</t>
+          <t>2027-11-01</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>CW30/27</t>
+          <t>CW44/27</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>CW21/27</t>
+          <t>CW35/27</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>1200</v>
+        <v>1588</v>
       </c>
     </row>
     <row r="25">
@@ -1486,25 +1486,25 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>960</v>
+        <v>1920</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2027-10-01</t>
+          <t>2028-01-01</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>CW39/27</t>
+          <t>CW52/27</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>CW30/27</t>
+          <t>CW43/27</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>960</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="26">
@@ -1529,25 +1529,25 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>960</v>
+        <v>1200</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2027-12-01</t>
+          <t>2028-03-01</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>CW48/27</t>
+          <t>CW09/28</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>CW39/27</t>
+          <t>CW52/27</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>572</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="27">
@@ -1576,451 +1576,21 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2027-12-01</t>
+          <t>2028-04-01</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>CW48/27</t>
+          <t>CW13/28</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>CW39/27</t>
+          <t>CW04/28</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER BRASIL</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>5441085</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>IR.3205-BD-2Z-3005&gt;A</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>1680</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>2028-01-01</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>CW52/27</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>CW43/27</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>1680</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER BRASIL</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>5441085</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>IR.3205-BD-2Z-3005&gt;A</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>480</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>2028-02-01</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>CW05/28</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>CW48/27</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER BRASIL</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>5441085</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>IR.3205-BD-2Z-3005&gt;A</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>1920</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2028-03-01</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>CW09/28</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>CW52/27</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>1920</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER BRASIL</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>5441085</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>IR.3205-BD-2Z-3005&gt;A</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>825</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>2028-05-01</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>CW18/28</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>CW09/28</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>825</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER PORTUGALLL</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>5500001822</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>F-804661-3005-A.IR.KL</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>3840</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>CW53/26</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>CW51/26</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>3468</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER PORTUGALLL</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>5500001822</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>F-804661-3005-A.IR.KL</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>3840</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>CW53/26</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>CW52/26</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER PORTUGAL</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>5500001822</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>F-804661-3005-A.IR.KL</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>3840</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>2027-02-22</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>CW08/27</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>CW06/27</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>1763</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER PORTUGAL</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>5500001822</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>F-804661-3005-A.IR.KL</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>3840</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>2027-02-22</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>CW08/27</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>CW06/27</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>2077</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER PORTUGAL</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>5500001822</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>F-804661-3005-A.IR.KL</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>3840</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>2027-04-19</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>CW16/27</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>CW14/27</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>3840</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>SCHAEFFLER PORTUGAL</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>5500001822</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>F-804661-3005-A.IR.KL</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>3840</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>2027-08-01</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>CW30/27</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>CW28/27</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>5</v>
+        <v>741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix to CSV import part.
</commit_message>
<xml_diff>
--- a/zlpi.xlsx
+++ b/zlpi.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -540,25 +540,25 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1536</v>
+        <v>3072</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CW47/26</t>
+          <t>CW09/27</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CW38/26</t>
+          <t>CW53/26</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1536</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="4">
@@ -583,25 +583,25 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3840</v>
+        <v>3072</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CW02/27</t>
+          <t>CW09/27</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CW46/26</t>
+          <t>CW53/26</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>3840</v>
+        <v>384</v>
       </c>
     </row>
     <row r="5">
@@ -626,25 +626,25 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3072</v>
+        <v>770</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CW09/27</t>
+          <t>CW44/26</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CW53/26</t>
+          <t>CW35/26</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>2688</v>
+        <v>770</v>
       </c>
     </row>
     <row r="6">
@@ -669,25 +669,25 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3072</v>
+        <v>771</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CW09/27</t>
+          <t>CW44/26</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CW53/26</t>
+          <t>CW35/26</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>384</v>
+        <v>771</v>
       </c>
     </row>
     <row r="7">
@@ -716,21 +716,21 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2027-04-23</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CW16/27</t>
+          <t>CW47/26</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CW07/27</t>
+          <t>CW38/26</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>616</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="8">
@@ -755,25 +755,25 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1536</v>
+        <v>3840</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2027-04-23</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CW16/27</t>
+          <t>CW02/27</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>CW07/27</t>
+          <t>CW46/26</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>920</v>
+        <v>2299</v>
       </c>
     </row>
     <row r="9">
@@ -802,21 +802,21 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2027-06-01</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>CW22/27</t>
+          <t>CW02/27</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>CW13/27</t>
+          <t>CW47/26</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>3840</v>
+        <v>616</v>
       </c>
     </row>
     <row r="10">
@@ -841,25 +841,25 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1536</v>
+        <v>3840</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2027-09-01</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>CW35/27</t>
+          <t>CW02/27</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>CW26/27</t>
+          <t>CW51/26</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>1536</v>
+        <v>925</v>
       </c>
     </row>
     <row r="11">
@@ -884,25 +884,25 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2304</v>
+        <v>1536</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2027-11-01</t>
+          <t>2027-02-22</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CW44/27</t>
+          <t>CW08/27</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CW35/27</t>
+          <t>CW52/26</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2304</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="12">
@@ -927,25 +927,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1536</v>
+        <v>2304</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2028-01-01</t>
+          <t>2027-04-19</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>CW52/27</t>
+          <t>CW16/27</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CW43/27</t>
+          <t>CW07/27</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1536</v>
+        <v>2304</v>
       </c>
     </row>
     <row r="13">
@@ -970,25 +970,25 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1536</v>
+        <v>4608</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2028-03-01</t>
+          <t>2027-06-01</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>CW09/28</t>
+          <t>CW22/27</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>CW52/27</t>
+          <t>CW13/27</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>1536</v>
+        <v>4608</v>
       </c>
     </row>
     <row r="14">
@@ -1013,25 +1013,25 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4663</v>
+        <v>2304</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2028-05-01</t>
+          <t>2027-10-01</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>CW18/28</t>
+          <t>CW39/27</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CW09/28</t>
+          <t>CW30/27</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2328</v>
+        <v>2304</v>
       </c>
     </row>
     <row r="15">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>5441085</t>
+          <t>5441084</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1052,29 +1052,29 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>IR.3205-BD-2Z-3005&gt;A</t>
+          <t>AU.3205-BD-2Z-3005-T</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>4080</v>
+        <v>2304</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-12-01</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CW02/27</t>
+          <t>CW48/27</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CW46/26</t>
+          <t>CW39/27</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>2351</v>
+        <v>2304</v>
       </c>
     </row>
     <row r="16">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>5441085</t>
+          <t>5441084</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1095,29 +1095,29 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IR.3205-BD-2Z-3005&gt;A</t>
+          <t>AU.3205-BD-2Z-3005-T</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>4080</v>
+        <v>768</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2028-02-01</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CW02/27</t>
+          <t>CW05/28</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>CW46/26</t>
+          <t>CW48/27</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>1729</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -1142,21 +1142,21 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>3360</v>
+        <v>4080</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CW09/27</t>
+          <t>CW02/27</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>CW53/26</t>
+          <t>CW46/26</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -1185,25 +1185,25 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3360</v>
+        <v>4080</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2027-03-01</t>
+          <t>2027-01-11</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>CW09/27</t>
+          <t>CW02/27</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>CW53/26</t>
+          <t>CW46/26</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>1009</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="19">
@@ -1228,25 +1228,25 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>720</v>
+        <v>3360</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2027-04-23</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CW16/27</t>
+          <t>CW09/27</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>CW07/27</t>
+          <t>CW53/26</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>720</v>
+        <v>2351</v>
       </c>
     </row>
     <row r="20">
@@ -1271,25 +1271,25 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2160</v>
+        <v>3360</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2027-06-01</t>
+          <t>2027-03-01</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>CW22/27</t>
+          <t>CW09/27</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CW13/27</t>
+          <t>CW53/26</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>2160</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="21">
@@ -1318,17 +1318,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2027-08-01</t>
+          <t>2027-04-23</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CW30/27</t>
+          <t>CW16/27</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CW21/27</t>
+          <t>CW07/27</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -1357,25 +1357,25 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1440</v>
+        <v>2160</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2027-09-01</t>
+          <t>2027-06-01</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>CW35/27</t>
+          <t>CW22/27</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CW26/27</t>
+          <t>CW13/27</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>1440</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="23">
@@ -1400,25 +1400,25 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1920</v>
+        <v>720</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2027-11-01</t>
+          <t>2027-08-01</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>CW44/27</t>
+          <t>CW30/27</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>CW35/27</t>
+          <t>CW21/27</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>332</v>
+        <v>720</v>
       </c>
     </row>
     <row r="24">
@@ -1443,25 +1443,25 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1920</v>
+        <v>1440</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2027-11-01</t>
+          <t>2027-09-01</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>CW44/27</t>
+          <t>CW35/27</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>CW35/27</t>
+          <t>CW26/27</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>1588</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="25">
@@ -1490,21 +1490,21 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2028-01-01</t>
+          <t>2027-11-01</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>CW52/27</t>
+          <t>CW44/27</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>CW43/27</t>
+          <t>CW35/27</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>1920</v>
+        <v>332</v>
       </c>
     </row>
     <row r="26">
@@ -1529,25 +1529,25 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>1200</v>
+        <v>1920</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2028-03-01</t>
+          <t>2027-11-01</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>CW09/28</t>
+          <t>CW44/27</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>CW52/27</t>
+          <t>CW35/27</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>1200</v>
+        <v>1588</v>
       </c>
     </row>
     <row r="27">
@@ -1572,25 +1572,326 @@
         </is>
       </c>
       <c r="E27" t="n">
+        <v>1920</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2028-01-01</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>CW52/27</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>CW43/27</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>1920</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER BRASIL</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>5441085</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>IR.3205-BD-2Z-3005&gt;A</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2028-03-01</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>CW09/28</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>CW52/27</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER BRASIL</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>5441085</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>IR.3205-BD-2Z-3005&gt;A</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
         <v>960</v>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>2028-04-01</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>CW13/28</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>CW04/28</t>
         </is>
       </c>
-      <c r="I27" t="n">
+      <c r="I29" t="n">
         <v>741</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER PORTUGAL</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>5500001822</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>F-804661-3005-A.IR.KL</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>3340</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>CW53/26</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>CW51/26</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>3340</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER PORTUGAL</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>5500001822</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>F-804661-3005-A.IR.KL</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>3840</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2027-02-22</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>CW08/27</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>CW06/27</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>3840</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER PORTUGAL</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>5500001822</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>F-804661-3005-A.IR.KL</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>3840</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2027-06-14</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>CW24/27</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>CW22/27</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>3840</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER PORTUGAL</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>5500001822</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>F-804661-3005-A.IR.KL</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>3840</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2027-10-01</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>CW39/27</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>CW37/27</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>3840</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>SCHAEFFLER PORTUGAL</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>5500001822</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>F-804661-3005-A.IR.KL</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>3840</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2027-10-25</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>CW43/27</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>CW41/27</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>